<commit_message>
docs: actualizar cronograma maestro de produccion v4
</commit_message>
<xml_diff>
--- a/docs/produccion/Cronograma_Maestro_Puesta_Produccion_MVS_Commerce.xlsx
+++ b/docs/produccion/Cronograma_Maestro_Puesta_Produccion_MVS_Commerce.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="1" r:id="R2849a20cc3b7484f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plan Producción" sheetId="2" r:id="R8d6e1406b75546bd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Centro de Datos" sheetId="3" r:id="R237ee9c096f640a3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisiones aprobadas" sheetId="4" r:id="R385bbb654f5d4192"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint Agentes" sheetId="5" r:id="Rfed3ae6fa91246ac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="1" r:id="Rc68c2b07827240df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plan Producción" sheetId="2" r:id="Rca10abdd1e5842ae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Centro de Datos" sheetId="3" r:id="Re45bc18cf6894b94"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisiones aprobadas" sheetId="4" r:id="R91f91f2cda2742fd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint Agentes" sheetId="5" r:id="Ra1d9aa702a704cf4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -81,7 +81,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="44">
+  <x:cellXfs count="45">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -178,6 +178,7 @@
     <x:xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -188,7 +189,7 @@
         <x:b/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDCFCE7"/>
         </x:patternFill>
       </x:fill>
@@ -198,7 +199,7 @@
         <x:b/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEF3C7"/>
         </x:patternFill>
       </x:fill>
@@ -208,14 +209,14 @@
         <x:b/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE0E7FF"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF8FAFC"/>
         </x:patternFill>
       </x:fill>
@@ -225,7 +226,7 @@
         <x:b/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE0E7FF"/>
         </x:patternFill>
       </x:fill>
@@ -235,21 +236,21 @@
         <x:b/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDCFCE7"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEF3C7"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE0E7FF"/>
         </x:patternFill>
       </x:fill>
@@ -1053,13 +1054,13 @@
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="36" t="str">
-        <x:v>P07</x:v>
+        <x:v>P07A</x:v>
       </x:c>
       <x:c r="B9" s="36" t="str">
         <x:v>Cliente</x:v>
       </x:c>
       <x:c r="C9" s="36" t="str">
-        <x:v>Portal personal del cliente</x:v>
+        <x:v>Portal de Clientes — experiencia del cliente</x:v>
       </x:c>
       <x:c r="D9" s="36" t="str">
         <x:v>PENDIENTE</x:v>
@@ -1071,65 +1072,65 @@
         <x:v>P06</x:v>
       </x:c>
       <x:c r="G9" s="36" t="str">
-        <x:v>Dar acceso privado al cliente a su fidelización.</x:v>
+        <x:v>Dar al cliente un portal privado, útil y comercial ligado a su empresa.</x:v>
       </x:c>
       <x:c r="H9" s="36" t="str">
-        <x:v>Auditar primero lo ya construido. Usuario + contraseña; cada cliente solo ve su información; saldo, movimientos, premios/beneficios, datos básicos y QR/link cuando aplique. Comprobantes pueden añadirse si ya hay base segura.</x:v>
+        <x:v>Scope obligatorio por company_id, nunca por sucursal. Usuario + contraseña y recuperación. Saldo consolidado de puntos de todas las sucursales; movimientos muestran sucursal de origen. Mostrar valor aproximado, mínimo de canje, puntos ganados/usados, fecha exacta y tiempo restante para vencimiento; una compra refleja renovación/extensión solo según la regla real de Fidelización. Premios, compras, comprobantes/PDF, perfil, Nuevos productos, Ofertas, Promociones, Avisos, 'Te falta poco' y 'Para ti'. CTA configurables por empresa: Comprar ahora / Tienda / Catálogo / WhatsApp. MYM podrá usar mymenlinea.com, nunca hardcodeado.</x:v>
       </x:c>
       <x:c r="I9" s="36" t="str">
-        <x:v>Autenticación, recuperación, aislamiento cliente/empresa, móvil, puntos/kardex.</x:v>
+        <x:v>Auth/recuperación; aislamiento empresa; cliente compra en 2 sucursales y ve saldo único; vigencia coincide con regla real; compras/comprobantes; publicaciones; CTA por empresa; 360/768/1280.</x:v>
       </x:c>
       <x:c r="J9" s="36" t="str">
-        <x:v>Cliente consulta su información sin exposición de terceros.</x:v>
+        <x:v>Portal único por empresa, seguro, consolidado y con contenido/acciones comerciales útiles.</x:v>
       </x:c>
       <x:c r="K9" s="36" t="str">
-        <x:v>feat: crear portal cliente P07</x:v>
+        <x:v>feat: crear portal clientes P07A</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="36" t="str">
-        <x:v>P08</x:v>
+        <x:v>P07B</x:v>
       </x:c>
       <x:c r="B10" s="36" t="str">
-        <x:v>Infraestructura</x:v>
+        <x:v>Fidelización</x:v>
       </x:c>
       <x:c r="C10" s="36" t="str">
-        <x:v>Dominio + servidor provisional + backups</x:v>
+        <x:v>Gestión de Portal de Clientes</x:v>
       </x:c>
       <x:c r="D10" s="36" t="str">
         <x:v>PENDIENTE</x:v>
       </x:c>
       <x:c r="E10" s="36" t="str">
-        <x:v>P0</x:v>
+        <x:v>P1</x:v>
       </x:c>
       <x:c r="F10" s="36" t="str">
-        <x:v>P03</x:v>
+        <x:v>P07A</x:v>
       </x:c>
       <x:c r="G10" s="36" t="str">
-        <x:v>Permitir acceso estable de San Ramón y Liberia antes del VPS definitivo.</x:v>
+        <x:v>Dar a cada empresa una administración simple de su portal y promociones desde Fidelización.</x:v>
       </x:c>
       <x:c r="H10" s="36" t="str">
-        <x:v>Preparar mvscommerce.com/app.mvscommerce.com cuando se compre; HTTPS estable; PC de San Ramón como servidor provisional; sin suspensión; arranque servicios; backup automático; recuperación documentada. Luego migrable a VPS.</x:v>
+        <x:v>Debe aparecer en el SIDEBAR dentro de Fidelización con nombre profesional 'Portal de Clientes'. NO pertenece al Panel Maestro/Superadmin. Dentro: Dashboard/Resumen, Publicaciones, Productos destacados, Enlaces y botones, Configuración y Vista previa. Crear/editar/eliminar/programar publicaciones; tipos Nuevo producto / Oferta / Promoción / Aviso; seleccionar producto real opcional; reutilizar imagen/nombre/precio/special_price; imagen propia opcional; mensaje; vigencia; activar/desactivar; ordenar/destacar; vista previa; opción de ofertas automáticas. Configurar uno o varios CTA por empresa: tienda/web, página de compra, catálogo WhatsApp, WhatsApp u otro enlace válido. Permisos granulares: administrar portal/configuración, gestionar publicaciones/promociones, gestionar enlaces y ver/vista previa. La empresa puede autorizar a Cajero o Vendedor a crear/publicar promociones sin darles configuración completa. Reutilizar roles/permisos existentes; no crear módulo Vendedores solo por esto.</x:v>
       </x:c>
       <x:c r="I10" s="36" t="str">
-        <x:v>Acceso remoto, reinicio, caída internet, restore backup, HTTPS, seguridad.</x:v>
+        <x:v>Permisos por rol/usuario; cajero autorizado publica pero no cambia configuración/enlaces si no tiene permiso; usuario sin permiso bloqueado; aislamiento empresa; CRUD/vigencia; producto real; CTA; vista previa; sidebar Fidelización; 360/768/1280.</x:v>
       </x:c>
       <x:c r="J10" s="36" t="str">
-        <x:v>Dos sucursales acceden establemente y existe recuperación probada.</x:v>
+        <x:v>Cada empresa administra su propio portal desde Fidelización con permisos granulares y sin intervención del Superadmin.</x:v>
       </x:c>
       <x:c r="K10" s="36" t="str">
-        <x:v>chore: preparar infraestructura produccion P08</x:v>
+        <x:v>feat: administrar portal clientes P07B</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="36" t="str">
-        <x:v>P09</x:v>
+        <x:v>P08</x:v>
       </x:c>
       <x:c r="B11" s="36" t="str">
-        <x:v>Implementación</x:v>
+        <x:v>Infraestructura</x:v>
       </x:c>
       <x:c r="C11" s="36" t="str">
-        <x:v>Crear MYM Beauty Center + 2 sucursales</x:v>
+        <x:v>Dominio + servidor provisional + backups</x:v>
       </x:c>
       <x:c r="D11" s="36" t="str">
         <x:v>PENDIENTE</x:v>
@@ -1138,33 +1139,33 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="F11" s="36" t="str">
-        <x:v>P03,P08</x:v>
+        <x:v>P03</x:v>
       </x:c>
       <x:c r="G11" s="36" t="str">
-        <x:v>Crear primera empresa real usando el mismo onboarding del producto.</x:v>
+        <x:v>Permitir acceso estable de San Ramón y Liberia antes del VPS definitivo.</x:v>
       </x:c>
       <x:c r="H11" s="36" t="str">
-        <x:v>Empresa MYM Beauty Center; sucursales San Ramón y Liberia; administradores/usuarios, cajas, métodos de pago, módulos y configuración. No hardcodear MYM en aplicación.</x:v>
+        <x:v>Preparar mvscommerce.com/app.mvscommerce.com cuando se compre; HTTPS estable; PC de San Ramón como servidor provisional; sin suspensión; arranque servicios; backup automático; recuperación documentada. Luego migrable a VPS.</x:v>
       </x:c>
       <x:c r="I11" s="36" t="str">
-        <x:v>Aislamiento, sucursales, permisos, cajas, configuración, acceso remoto.</x:v>
+        <x:v>Acceso remoto, reinicio, caída internet, restore backup, HTTPS, seguridad.</x:v>
       </x:c>
       <x:c r="J11" s="36" t="str">
-        <x:v>MYM existe como tenant real y ambas sucursales operan separadas.</x:v>
+        <x:v>Dos sucursales acceden establemente y existe recuperación probada.</x:v>
       </x:c>
       <x:c r="K11" s="36" t="str">
-        <x:v>chore: configurar MYM produccion P09</x:v>
+        <x:v>chore: preparar infraestructura produccion P08</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="36" t="str">
-        <x:v>P10</x:v>
+        <x:v>P09</x:v>
       </x:c>
       <x:c r="B12" s="36" t="str">
-        <x:v>Salida</x:v>
+        <x:v>Implementación</x:v>
       </x:c>
       <x:c r="C12" s="36" t="str">
-        <x:v>Ensayo de migración + piloto productivo</x:v>
+        <x:v>Crear MYM Beauty Center + 2 sucursales</x:v>
       </x:c>
       <x:c r="D12" s="36" t="str">
         <x:v>PENDIENTE</x:v>
@@ -1173,56 +1174,91 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="F12" s="36" t="str">
+        <x:v>P03,P08</x:v>
+      </x:c>
+      <x:c r="G12" s="36" t="str">
+        <x:v>Crear primera empresa real usando el mismo onboarding del producto.</x:v>
+      </x:c>
+      <x:c r="H12" s="36" t="str">
+        <x:v>Empresa MYM Beauty Center; sucursales San Ramón y Liberia; administradores/usuarios, cajas, métodos de pago, módulos y configuración. No hardcodear MYM en aplicación.</x:v>
+      </x:c>
+      <x:c r="I12" s="36" t="str">
+        <x:v>Aislamiento, sucursales, permisos, cajas, configuración, acceso remoto.</x:v>
+      </x:c>
+      <x:c r="J12" s="36" t="str">
+        <x:v>MYM existe como tenant real y ambas sucursales operan separadas.</x:v>
+      </x:c>
+      <x:c r="K12" s="36" t="str">
+        <x:v>chore: configurar MYM produccion P09</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="36" t="str">
+        <x:v>P10</x:v>
+      </x:c>
+      <x:c r="B13" s="36" t="str">
+        <x:v>Salida</x:v>
+      </x:c>
+      <x:c r="C13" s="36" t="str">
+        <x:v>Ensayo de migración + piloto productivo</x:v>
+      </x:c>
+      <x:c r="D13" s="36" t="str">
+        <x:v>PENDIENTE</x:v>
+      </x:c>
+      <x:c r="E13" s="36" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="F13" s="36" t="str">
         <x:v>P09,D04,D05,D06,D07,D08,D09</x:v>
       </x:c>
-      <x:c r="G12" s="36" t="str">
+      <x:c r="G13" s="36" t="str">
         <x:v>Migrar con seguridad y comenzar a producir.</x:v>
       </x:c>
-      <x:c r="H12" s="36" t="str">
+      <x:c r="H13" s="36" t="str">
         <x:v>Primero ensayo con copia; luego corte final. Prioridad: productos/códigos, clientes, proveedores, inventario por sucursal, CxC/CxP, puntos, usuarios/configuración. Históricos no bloquean salida salvo decisión expresa.</x:v>
       </x:c>
-      <x:c r="I12" s="36" t="str">
+      <x:c r="I13" s="36" t="str">
         <x:v>Conciliación origen/MVS, venta real, caja, inventario, cliente, fidelización, impresión, correo, backup/restore.</x:v>
       </x:c>
-      <x:c r="J12" s="36" t="str">
+      <x:c r="J13" s="36" t="str">
         <x:v>Piloto aprobado y diferencias documentadas/cero críticas.</x:v>
       </x:c>
-      <x:c r="K12" s="36" t="str">
+      <x:c r="K13" s="36" t="str">
         <x:v>test: validar piloto produccion P10</x:v>
       </x:c>
     </x:row>
-    <x:row r="13">
-      <x:c r="A13" t="str">
+    <x:row r="14">
+      <x:c r="A14" s="36" t="str">
         <x:v>V02</x:v>
       </x:c>
-      <x:c r="B13" t="str">
+      <x:c r="B14" s="36" t="str">
         <x:v>Evolución</x:v>
       </x:c>
-      <x:c r="C13" t="str">
+      <x:c r="C14" s="36" t="str">
         <x:v>Wallet móvil del cliente</x:v>
       </x:c>
-      <x:c r="D13" t="str">
+      <x:c r="D14" s="36" t="str">
         <x:v>POST-MVP</x:v>
       </x:c>
-      <x:c r="E13" t="str">
+      <x:c r="E14" s="36" t="str">
         <x:v>P2</x:v>
       </x:c>
-      <x:c r="F13" t="str">
-        <x:v>P07</x:v>
-      </x:c>
-      <x:c r="G13" t="str">
+      <x:c r="F14" s="36" t="str">
+        <x:v>P07A</x:v>
+      </x:c>
+      <x:c r="G14" s="36" t="str">
         <x:v>Evaluar pase/tarjeta de fidelización en wallets móviles.</x:v>
       </x:c>
-      <x:c r="H13" t="str">
+      <x:c r="H14" s="36" t="str">
         <x:v>Apple Wallet y Samsung Wallet/equivalente. No bloquea la salida inicial. Diseñar cuando portal/QR estén estables.</x:v>
       </x:c>
-      <x:c r="I13" t="str">
+      <x:c r="I14" s="36" t="str">
         <x:v>Compatibilidad, seguridad del pase, actualización de saldo, revocación.</x:v>
       </x:c>
-      <x:c r="J13" t="str">
+      <x:c r="J14" s="36" t="str">
         <x:v>Decisión técnica y comercial aprobada para V0.2.</x:v>
       </x:c>
-      <x:c r="K13" t="str">
+      <x:c r="K14" s="36" t="str">
         <x:v>feat: integrar wallet cliente V02</x:v>
       </x:c>
     </x:row>
@@ -1627,10 +1663,10 @@
         <x:v>Portal cliente</x:v>
       </x:c>
       <x:c r="B7" s="36" t="str">
-        <x:v>Acceso personal con usuario y contraseña; aislamiento; puntos/movimientos/premios/datos; QR/link cuando aplique.</x:v>
+        <x:v>Acceso personal con usuario y contraseña; scope por EMPRESA, no sucursal. Consolida puntos/compras de todas las sucursales y conserva origen por movimiento. Mostrar fecha y tiempo restante para vencimiento de puntos y actualizar vigencia tras compras solo según la regla real de Fidelización. Portal MVP: puntos, mínimo/valor, movimientos, premios, compras, comprobantes, perfil, Nuevos productos, Ofertas, Promociones y Avisos. La empresa configura CTA comerciales (web/tienda/página de compra/catálogo WhatsApp/WhatsApp) y las publicaciones reutilizan el catálogo real.</x:v>
       </x:c>
       <x:c r="C7" s="36" t="str">
-        <x:v>No exponer datos de otros clientes o empresas.</x:v>
+        <x:v>No ligar acceso/saldo a branch_id. No inventar otra regla de vencimiento. No mezclar empresas. No hardcodear mymenlinea.com. No duplicar catálogo. No convertir P07 en e-commerce completo ni exigir IA/Wallet en MVP.</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -1675,6 +1711,39 @@
       </x:c>
       <x:c r="C11" s="36" t="str">
         <x:v>No dos agentes tocando simultáneamente los mismos archivos.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="36" t="str">
+        <x:v>Contenido del portal</x:v>
+      </x:c>
+      <x:c r="B12" s="36" t="str">
+        <x:v>La empresa tendrá una administración simple de publicaciones: tipo (Nuevo producto / Oferta / Promoción / Aviso), producto opcional, imagen, mensaje, vigencia y Publicar. Ofertas del catálogo pueden mostrarse automáticamente si están activas.</x:v>
+      </x:c>
+      <x:c r="C12" s="36" t="str">
+        <x:v>No convertir P07 en e-commerce completo; carrito/compra online, push, IA avanzada y Wallet quedan fuera del MVP.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="36" t="str">
+        <x:v>Enlaces comerciales del portal</x:v>
+      </x:c>
+      <x:c r="B13" s="36" t="str">
+        <x:v>Cada empresa puede configurar uno o varios CTA del portal: Comprar ahora, Ver tienda, Ver catálogo o WhatsApp. El destino puede ser web/e-commerce, página de compra, catálogo de WhatsApp o enlace comercial. MYM podrá apuntar a mymenlinea.com, pero la plataforma debe ser genérica para cualquier empresa.</x:v>
+      </x:c>
+      <x:c r="C13" s="36" t="str">
+        <x:v>No fijar URLs de MYM en código ni obligar a todas las empresas a tener e-commerce.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="36" t="str">
+        <x:v>Permisos Portal de Clientes</x:v>
+      </x:c>
+      <x:c r="B14" s="36" t="str">
+        <x:v>Portal de Clientes vive dentro de Fidelización y es interno de cada empresa. Usar permisos granulares para separar configuración, publicaciones/promociones, enlaces y consulta/vista previa. Cajero o Vendedor pueden recibir permiso para crear/publicar promociones sin obtener administración completa. Los roles son configurables por la empresa.</x:v>
+      </x:c>
+      <x:c r="C14" s="36" t="str">
+        <x:v>No administrar contenido del portal desde el Panel Maestro MVS. No asumir que todo cajero publica por defecto. No crear un módulo separado de Vendedores para este alcance.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1812,22 +1881,22 @@
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="36" t="str">
-        <x:v>S4</x:v>
+        <x:v>S4A</x:v>
       </x:c>
       <x:c r="B6" s="36" t="str">
-        <x:v>P07 Portal cliente</x:v>
+        <x:v>P07A Portal de Clientes</x:v>
       </x:c>
       <x:c r="C6" s="36" t="str">
         <x:v>Codex / MiMo relevo</x:v>
       </x:c>
       <x:c r="D6" s="36" t="str">
-        <x:v>Sí tras auditoría</x:v>
+        <x:v>Sí tras auditoría: portal por company_id, auth, puntos/vigencia, compras/comprobantes, contenido y CTA.</x:v>
       </x:c>
       <x:c r="E6" s="36" t="str">
-        <x:v>Autenticación/aislamiento no claro</x:v>
+        <x:v>Autenticación/aislamiento no claro o necesidad de e-commerce/Wallet/IA avanzada.</x:v>
       </x:c>
       <x:c r="F6" s="36" t="str">
-        <x:v>Sí, P07</x:v>
+        <x:v>Sí, P07A</x:v>
       </x:c>
       <x:c r="G6" s="36" t="str">
         <x:v>PENDIENTE</x:v>
@@ -1835,22 +1904,22 @@
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="36" t="str">
-        <x:v>S5</x:v>
+        <x:v>S4B</x:v>
       </x:c>
       <x:c r="B7" s="36" t="str">
-        <x:v>D04–D08 Migradores</x:v>
+        <x:v>P07B Gestión Portal de Clientes</x:v>
       </x:c>
       <x:c r="C7" s="36" t="str">
-        <x:v>Codex</x:v>
+        <x:v>Codex / MiMo relevo</x:v>
       </x:c>
       <x:c r="D7" s="36" t="str">
-        <x:v>Solo con plantillas MYM aprobadas</x:v>
+        <x:v>Sí: administración dentro de Fidelización, permisos granulares, publicaciones, enlaces y vista previa.</x:v>
       </x:c>
       <x:c r="E7" s="36" t="str">
-        <x:v>Falta plantilla o columna no mapeada</x:v>
+        <x:v>Conflicto con roles/permisos existentes o alcance requiere nuevo módulo comercial.</x:v>
       </x:c>
       <x:c r="F7" s="36" t="str">
-        <x:v>Sí, uno por fase</x:v>
+        <x:v>Sí, P07B</x:v>
       </x:c>
       <x:c r="G7" s="36" t="str">
         <x:v>PENDIENTE</x:v>

</xml_diff>